<commit_message>
chore: update teacher schedule template and bump version to v1.617
</commit_message>
<xml_diff>
--- a/Template_Horario_Maestro.xlsx
+++ b/Template_Horario_Maestro.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rmartin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\Customers\CBTis73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569CD0BE-3FF7-4334-BF99-94A0E0037824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D0B559-8E3B-4744-99BD-CDF73E6461DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1066DCBB-7658-485D-B378-A5A8C35F949C}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23596" windowHeight="15076" xr2:uid="{1066DCBB-7658-485D-B378-A5A8C35F949C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="97">
   <si>
     <t>Horas</t>
   </si>
@@ -200,18 +200,6 @@
     <t>CLAVE</t>
   </si>
   <si>
-    <t>LUNES</t>
-  </si>
-  <si>
-    <t>MARTES</t>
-  </si>
-  <si>
-    <t>JUEVES</t>
-  </si>
-  <si>
-    <t>VIERNES</t>
-  </si>
-  <si>
     <t>HORARIO TURNO VESPERTINO</t>
   </si>
   <si>
@@ -225,9 +213,6 @@
   </si>
   <si>
     <t>la DGETI</t>
-  </si>
-  <si>
-    <t>MIERC.</t>
   </si>
   <si>
     <t>Yolanda Morales Miranda</t>
@@ -1169,7 +1154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1405,15 +1390,60 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1429,95 +1459,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1964,24 +1913,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58F58D38-BD95-48DF-854F-C3512D201DF1}">
   <dimension ref="A4:AT58"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.73046875" defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" customWidth="1"/>
-    <col min="5" max="5" width="37.140625" customWidth="1"/>
-    <col min="6" max="6" width="6.28515625" customWidth="1"/>
-    <col min="7" max="7" width="4.42578125" customWidth="1"/>
+    <col min="1" max="1" width="4.3984375" customWidth="1"/>
+    <col min="2" max="2" width="9.73046875" customWidth="1"/>
+    <col min="3" max="3" width="12.3984375" customWidth="1"/>
+    <col min="5" max="5" width="37.1328125" customWidth="1"/>
+    <col min="6" max="6" width="6.265625" customWidth="1"/>
+    <col min="7" max="7" width="4.3984375" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="13" width="8.85546875" customWidth="1"/>
-    <col min="14" max="14" width="6.7109375" customWidth="1"/>
-    <col min="15" max="17" width="9.7109375" customWidth="1"/>
-    <col min="18" max="18" width="9.42578125" customWidth="1"/>
+    <col min="9" max="13" width="8.86328125" customWidth="1"/>
+    <col min="14" max="14" width="6.73046875" customWidth="1"/>
+    <col min="15" max="17" width="9.73046875" customWidth="1"/>
+    <col min="18" max="18" width="9.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:46" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:46" ht="15" x14ac:dyDescent="0.35">
       <c r="B4" s="56" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C4" s="56"/>
       <c r="D4" s="56"/>
@@ -1999,9 +1948,9 @@
       <c r="P4" s="56"/>
       <c r="Q4" s="56"/>
     </row>
-    <row r="5" spans="1:46" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:46" ht="15" x14ac:dyDescent="0.35">
       <c r="B5" s="56" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C5" s="56"/>
       <c r="D5" s="56"/>
@@ -2019,9 +1968,9 @@
       <c r="P5" s="56"/>
       <c r="Q5" s="56"/>
     </row>
-    <row r="6" spans="1:46" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:46" ht="15" x14ac:dyDescent="0.35">
       <c r="B6" s="56" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C6" s="56"/>
       <c r="D6" s="56"/>
@@ -2039,7 +1988,7 @@
       <c r="P6" s="56"/>
       <c r="Q6" s="56"/>
     </row>
-    <row r="7" spans="1:46" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:46" ht="15" x14ac:dyDescent="0.35">
       <c r="B7" s="56"/>
       <c r="C7" s="56"/>
       <c r="D7" s="56"/>
@@ -2057,7 +2006,7 @@
       <c r="P7" s="56"/>
       <c r="Q7" s="56"/>
     </row>
-    <row r="8" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -2076,7 +2025,7 @@
       <c r="AB8" s="4"/>
       <c r="AC8" s="4"/>
     </row>
-    <row r="9" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B9" s="6" t="s">
         <v>18</v>
       </c>
@@ -2120,7 +2069,7 @@
       <c r="AB9" s="4"/>
       <c r="AC9" s="4"/>
     </row>
-    <row r="10" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B10" s="11" t="s">
         <v>19</v>
       </c>
@@ -2177,7 +2126,7 @@
       <c r="AS10" s="4"/>
       <c r="AT10" s="4"/>
     </row>
-    <row r="11" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B11" s="13"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
@@ -2195,7 +2144,7 @@
       <c r="P11" s="5"/>
       <c r="Q11" s="12"/>
     </row>
-    <row r="12" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="14" t="s">
         <v>24</v>
       </c>
@@ -2217,7 +2166,7 @@
       <c r="P12" s="8"/>
       <c r="Q12" s="16"/>
     </row>
-    <row r="13" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="14" t="s">
         <v>26</v>
       </c>
@@ -2226,13 +2175,13 @@
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
       <c r="G13" s="15" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
       <c r="K13" s="15" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="L13" s="8"/>
       <c r="M13" s="8"/>
@@ -2241,7 +2190,7 @@
       <c r="P13" s="8"/>
       <c r="Q13" s="16"/>
     </row>
-    <row r="14" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="4"/>
       <c r="B14" s="14" t="s">
         <v>27</v>
@@ -2254,7 +2203,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
       <c r="H14" s="15" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
@@ -2266,7 +2215,7 @@
       <c r="P14" s="8"/>
       <c r="Q14" s="16"/>
     </row>
-    <row r="15" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:46" x14ac:dyDescent="0.35">
       <c r="B15" s="17" t="s">
         <v>31</v>
       </c>
@@ -2288,7 +2237,7 @@
       <c r="P15" s="9"/>
       <c r="Q15" s="24"/>
     </row>
-    <row r="16" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:46" x14ac:dyDescent="0.35">
       <c r="B16" s="25" t="s">
         <v>30</v>
       </c>
@@ -2307,16 +2256,16 @@
         <v>29</v>
       </c>
       <c r="K16" s="28"/>
-      <c r="L16" s="104" t="s">
+      <c r="L16" s="119" t="s">
         <v>49</v>
       </c>
-      <c r="M16" s="105"/>
-      <c r="N16" s="105"/>
-      <c r="O16" s="105"/>
-      <c r="P16" s="105"/>
-      <c r="Q16" s="106"/>
-    </row>
-    <row r="17" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M16" s="120"/>
+      <c r="N16" s="120"/>
+      <c r="O16" s="120"/>
+      <c r="P16" s="120"/>
+      <c r="Q16" s="121"/>
+    </row>
+    <row r="17" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B17" s="25" t="s">
         <v>32</v>
       </c>
@@ -2348,12 +2297,12 @@
       <c r="P17" s="5"/>
       <c r="Q17" s="12"/>
     </row>
-    <row r="18" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B18" s="32" t="s">
         <v>33</v>
       </c>
       <c r="C18" s="55" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D18" s="26" t="s">
         <v>39</v>
@@ -2379,7 +2328,7 @@
       <c r="Q18" s="16"/>
       <c r="S18" s="3"/>
     </row>
-    <row r="19" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B19" s="44"/>
       <c r="C19" s="45"/>
       <c r="D19" s="19"/>
@@ -2388,8 +2337,8 @@
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
-      <c r="J19" s="110"/>
-      <c r="K19" s="111"/>
+      <c r="J19" s="108"/>
+      <c r="K19" s="124"/>
       <c r="L19" s="15"/>
       <c r="M19" s="60"/>
       <c r="N19" s="54"/>
@@ -2397,7 +2346,7 @@
       <c r="P19" s="60"/>
       <c r="Q19" s="16"/>
     </row>
-    <row r="20" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B20" s="36"/>
       <c r="C20" s="37"/>
       <c r="D20" s="37"/>
@@ -2415,7 +2364,7 @@
       <c r="P20" s="8"/>
       <c r="Q20" s="16"/>
     </row>
-    <row r="21" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B21" s="36"/>
       <c r="C21" s="37"/>
       <c r="D21" s="37"/>
@@ -2433,7 +2382,7 @@
       <c r="P21" s="8"/>
       <c r="Q21" s="16"/>
     </row>
-    <row r="22" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B22" s="36"/>
       <c r="C22" s="37"/>
       <c r="D22" s="37"/>
@@ -2451,7 +2400,7 @@
       <c r="P22" s="8"/>
       <c r="Q22" s="16"/>
     </row>
-    <row r="23" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B23" s="38"/>
       <c r="C23" s="39"/>
       <c r="D23" s="39"/>
@@ -2470,7 +2419,7 @@
       <c r="Q23" s="12"/>
       <c r="R23" s="53"/>
     </row>
-    <row r="24" spans="2:23" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:23" x14ac:dyDescent="0.35">
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
@@ -2490,7 +2439,7 @@
       <c r="R24" s="53"/>
       <c r="W24" s="2"/>
     </row>
-    <row r="25" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B25" s="9" t="s">
         <v>16</v>
       </c>
@@ -2511,21 +2460,21 @@
       <c r="Q25" s="9"/>
       <c r="R25" s="53"/>
     </row>
-    <row r="26" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
-      <c r="H26" s="112" t="s">
+      <c r="H26" s="125" t="s">
         <v>11</v>
       </c>
-      <c r="I26" s="109"/>
-      <c r="J26" s="109"/>
-      <c r="K26" s="109"/>
-      <c r="L26" s="109"/>
-      <c r="M26" s="113"/>
+      <c r="I26" s="116"/>
+      <c r="J26" s="116"/>
+      <c r="K26" s="116"/>
+      <c r="L26" s="116"/>
+      <c r="M26" s="117"/>
       <c r="N26" s="9"/>
       <c r="O26" s="71"/>
       <c r="P26" s="40" t="s">
@@ -2534,17 +2483,17 @@
       <c r="Q26" s="72"/>
       <c r="R26" s="53"/>
     </row>
-    <row r="27" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B27" s="73" t="s">
         <v>53</v>
       </c>
       <c r="C27" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="D27" s="109" t="s">
+      <c r="D27" s="116" t="s">
         <v>52</v>
       </c>
-      <c r="E27" s="109"/>
+      <c r="E27" s="116"/>
       <c r="F27" s="75" t="s">
         <v>36</v>
       </c>
@@ -2568,153 +2517,141 @@
         <v>10</v>
       </c>
       <c r="N27" s="9"/>
-      <c r="O27" s="14" t="s">
-        <v>54</v>
-      </c>
+      <c r="O27" s="14"/>
       <c r="P27" s="57"/>
       <c r="Q27" s="58"/>
       <c r="R27" s="53"/>
     </row>
-    <row r="28" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B28" s="67"/>
       <c r="C28" s="68"/>
-      <c r="D28" s="107"/>
-      <c r="E28" s="108"/>
+      <c r="D28" s="122"/>
+      <c r="E28" s="123"/>
       <c r="F28" s="74"/>
       <c r="G28" s="9"/>
       <c r="H28" s="89" t="s">
-        <v>83</v>
-      </c>
-      <c r="I28" s="128"/>
-      <c r="J28" s="129"/>
-      <c r="K28" s="130"/>
-      <c r="L28" s="129"/>
-      <c r="M28" s="131"/>
+        <v>78</v>
+      </c>
+      <c r="I28" s="97"/>
+      <c r="J28" s="84"/>
+      <c r="K28" s="49"/>
+      <c r="L28" s="84"/>
+      <c r="M28" s="85"/>
       <c r="N28" s="9"/>
-      <c r="O28" s="14" t="s">
-        <v>54</v>
-      </c>
+      <c r="O28" s="14"/>
       <c r="P28" s="57"/>
       <c r="Q28" s="58"/>
       <c r="R28" s="53"/>
     </row>
-    <row r="29" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B29" s="67"/>
       <c r="C29" s="74"/>
-      <c r="D29" s="102"/>
-      <c r="E29" s="103"/>
-      <c r="F29" s="127"/>
+      <c r="D29" s="104"/>
+      <c r="E29" s="105"/>
+      <c r="F29" s="74"/>
       <c r="G29" s="9"/>
       <c r="H29" s="90" t="s">
-        <v>84</v>
-      </c>
-      <c r="I29" s="132"/>
-      <c r="J29" s="133"/>
-      <c r="K29" s="129"/>
-      <c r="L29" s="133"/>
-      <c r="M29" s="134"/>
+        <v>79</v>
+      </c>
+      <c r="I29" s="46"/>
+      <c r="J29" s="42"/>
+      <c r="K29" s="84"/>
+      <c r="L29" s="42"/>
+      <c r="M29" s="48"/>
       <c r="N29" s="9"/>
-      <c r="O29" s="14" t="s">
-        <v>55</v>
-      </c>
+      <c r="O29" s="14"/>
       <c r="P29" s="57"/>
       <c r="Q29" s="58"/>
       <c r="R29" s="53"/>
     </row>
-    <row r="30" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B30" s="67"/>
       <c r="C30" s="74"/>
-      <c r="D30" s="102"/>
-      <c r="E30" s="103"/>
-      <c r="F30" s="127"/>
+      <c r="D30" s="104"/>
+      <c r="E30" s="105"/>
+      <c r="F30" s="74"/>
       <c r="G30" s="9"/>
       <c r="H30" s="90" t="s">
-        <v>85</v>
-      </c>
-      <c r="I30" s="132"/>
-      <c r="J30" s="133"/>
-      <c r="K30" s="133"/>
-      <c r="L30" s="133"/>
-      <c r="M30" s="134"/>
+        <v>80</v>
+      </c>
+      <c r="I30" s="46"/>
+      <c r="J30" s="42"/>
+      <c r="K30" s="42"/>
+      <c r="L30" s="42"/>
+      <c r="M30" s="48"/>
       <c r="N30" s="9"/>
-      <c r="O30" s="14" t="s">
-        <v>63</v>
-      </c>
+      <c r="O30" s="14"/>
       <c r="P30" s="57"/>
       <c r="Q30" s="58"/>
       <c r="R30" s="53"/>
     </row>
-    <row r="31" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B31" s="47"/>
       <c r="C31" s="70"/>
-      <c r="D31" s="102"/>
-      <c r="E31" s="103"/>
+      <c r="D31" s="104"/>
+      <c r="E31" s="105"/>
       <c r="F31" s="69"/>
       <c r="G31" s="9"/>
       <c r="H31" s="91" t="s">
-        <v>86</v>
-      </c>
-      <c r="I31" s="122" t="s">
-        <v>77</v>
-      </c>
-      <c r="J31" s="123"/>
-      <c r="K31" s="123"/>
-      <c r="L31" s="123"/>
-      <c r="M31" s="124"/>
+        <v>81</v>
+      </c>
+      <c r="I31" s="101" t="s">
+        <v>72</v>
+      </c>
+      <c r="J31" s="102"/>
+      <c r="K31" s="102"/>
+      <c r="L31" s="102"/>
+      <c r="M31" s="103"/>
       <c r="N31" s="9"/>
-      <c r="O31" s="14" t="s">
-        <v>56</v>
-      </c>
+      <c r="O31" s="14"/>
       <c r="P31" s="57"/>
       <c r="Q31" s="58"/>
       <c r="R31" s="53"/>
     </row>
-    <row r="32" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B32" s="47"/>
       <c r="C32" s="70"/>
-      <c r="D32" s="102"/>
-      <c r="E32" s="103"/>
+      <c r="D32" s="104"/>
+      <c r="E32" s="105"/>
       <c r="F32" s="70"/>
       <c r="G32" s="9"/>
       <c r="H32" s="90" t="s">
-        <v>87</v>
-      </c>
-      <c r="I32" s="132"/>
-      <c r="J32" s="133"/>
-      <c r="K32" s="133"/>
-      <c r="L32" s="133"/>
-      <c r="M32" s="134"/>
+        <v>82</v>
+      </c>
+      <c r="I32" s="46"/>
+      <c r="J32" s="42"/>
+      <c r="K32" s="42"/>
+      <c r="L32" s="42"/>
+      <c r="M32" s="48"/>
       <c r="N32" s="9"/>
-      <c r="O32" s="14" t="s">
-        <v>57</v>
-      </c>
+      <c r="O32" s="14"/>
       <c r="P32" s="57"/>
       <c r="Q32" s="58"/>
       <c r="R32" s="53"/>
     </row>
-    <row r="33" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B33" s="47"/>
       <c r="C33" s="70"/>
-      <c r="D33" s="102"/>
-      <c r="E33" s="103"/>
+      <c r="D33" s="104"/>
+      <c r="E33" s="105"/>
       <c r="F33" s="70"/>
       <c r="G33" s="9"/>
       <c r="H33" s="90" t="s">
-        <v>88</v>
-      </c>
-      <c r="I33" s="132" t="s">
+        <v>83</v>
+      </c>
+      <c r="I33" s="46" t="s">
         <v>51</v>
       </c>
-      <c r="J33" s="133" t="s">
+      <c r="J33" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="K33" s="133" t="s">
+      <c r="K33" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="L33" s="133" t="s">
+      <c r="L33" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="M33" s="134" t="s">
+      <c r="M33" s="48" t="s">
         <v>51</v>
       </c>
       <c r="N33" s="9"/>
@@ -2723,69 +2660,69 @@
       <c r="Q33" s="58"/>
       <c r="R33" s="53"/>
     </row>
-    <row r="34" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B34" s="47"/>
       <c r="C34" s="70"/>
-      <c r="D34" s="118"/>
-      <c r="E34" s="119"/>
+      <c r="D34" s="112"/>
+      <c r="E34" s="113"/>
       <c r="F34" s="62"/>
       <c r="G34" s="9"/>
       <c r="H34" s="91" t="s">
-        <v>89</v>
-      </c>
-      <c r="I34" s="122" t="s">
-        <v>78</v>
-      </c>
-      <c r="J34" s="123"/>
-      <c r="K34" s="123"/>
-      <c r="L34" s="123"/>
-      <c r="M34" s="124"/>
+        <v>84</v>
+      </c>
+      <c r="I34" s="101" t="s">
+        <v>73</v>
+      </c>
+      <c r="J34" s="102"/>
+      <c r="K34" s="102"/>
+      <c r="L34" s="102"/>
+      <c r="M34" s="103"/>
       <c r="N34" s="9"/>
       <c r="O34" s="13"/>
-      <c r="P34" s="8"/>
+      <c r="P34" s="57"/>
       <c r="Q34" s="12"/>
     </row>
-    <row r="35" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B35" s="47"/>
       <c r="C35" s="70"/>
-      <c r="D35" s="120"/>
-      <c r="E35" s="103"/>
+      <c r="D35" s="114"/>
+      <c r="E35" s="105"/>
       <c r="F35" s="70"/>
       <c r="G35" s="9"/>
       <c r="H35" s="90" t="s">
-        <v>67</v>
-      </c>
-      <c r="I35" s="132"/>
-      <c r="J35" s="133"/>
-      <c r="K35" s="133"/>
-      <c r="L35" s="133"/>
-      <c r="M35" s="134"/>
+        <v>62</v>
+      </c>
+      <c r="I35" s="46"/>
+      <c r="J35" s="42"/>
+      <c r="K35" s="42"/>
+      <c r="L35" s="42"/>
+      <c r="M35" s="48"/>
       <c r="N35" s="9"/>
       <c r="O35" s="13"/>
-      <c r="P35" s="8"/>
+      <c r="P35" s="57"/>
       <c r="Q35" s="12"/>
     </row>
-    <row r="36" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B36" s="76"/>
       <c r="C36" s="77"/>
-      <c r="D36" s="125"/>
-      <c r="E36" s="126"/>
+      <c r="D36" s="106"/>
+      <c r="E36" s="107"/>
       <c r="F36" s="63"/>
       <c r="G36" s="9"/>
       <c r="H36" s="90" t="s">
-        <v>90</v>
-      </c>
-      <c r="I36" s="132"/>
-      <c r="J36" s="133"/>
-      <c r="K36" s="133"/>
-      <c r="L36" s="133"/>
-      <c r="M36" s="134"/>
+        <v>85</v>
+      </c>
+      <c r="I36" s="46"/>
+      <c r="J36" s="42"/>
+      <c r="K36" s="42"/>
+      <c r="L36" s="42"/>
+      <c r="M36" s="48"/>
       <c r="N36" s="9"/>
       <c r="O36" s="14"/>
-      <c r="P36" s="8"/>
+      <c r="P36" s="57"/>
       <c r="Q36" s="16"/>
     </row>
-    <row r="37" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B37" s="9" t="s">
         <v>4</v>
       </c>
@@ -2798,19 +2735,19 @@
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
       <c r="H37" s="90" t="s">
-        <v>91</v>
-      </c>
-      <c r="I37" s="132"/>
-      <c r="J37" s="133"/>
-      <c r="K37" s="133"/>
-      <c r="L37" s="133"/>
-      <c r="M37" s="134"/>
+        <v>86</v>
+      </c>
+      <c r="I37" s="46"/>
+      <c r="J37" s="42"/>
+      <c r="K37" s="42"/>
+      <c r="L37" s="42"/>
+      <c r="M37" s="48"/>
       <c r="N37" s="9"/>
       <c r="O37" s="14"/>
-      <c r="P37" s="8"/>
+      <c r="P37" s="57"/>
       <c r="Q37" s="16"/>
     </row>
-    <row r="38" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
@@ -2818,19 +2755,19 @@
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
       <c r="H38" s="89" t="s">
-        <v>92</v>
-      </c>
-      <c r="I38" s="135"/>
-      <c r="J38" s="136"/>
-      <c r="K38" s="136"/>
-      <c r="L38" s="136"/>
-      <c r="M38" s="137"/>
+        <v>87</v>
+      </c>
+      <c r="I38" s="79"/>
+      <c r="J38" s="80"/>
+      <c r="K38" s="80"/>
+      <c r="L38" s="80"/>
+      <c r="M38" s="81"/>
       <c r="N38" s="9"/>
       <c r="O38" s="14"/>
-      <c r="P38" s="8"/>
+      <c r="P38" s="57"/>
       <c r="Q38" s="16"/>
     </row>
-    <row r="39" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B39" s="9" t="s">
         <v>17</v>
       </c>
@@ -2841,7 +2778,7 @@
       <c r="G39" s="9"/>
       <c r="H39" s="92"/>
       <c r="I39" s="82" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="J39" s="82"/>
       <c r="K39" s="82"/>
@@ -2849,10 +2786,10 @@
       <c r="M39" s="83"/>
       <c r="N39" s="9"/>
       <c r="O39" s="14"/>
-      <c r="P39" s="8"/>
+      <c r="P39" s="57"/>
       <c r="Q39" s="16"/>
     </row>
-    <row r="40" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
       <c r="D40" s="9"/>
@@ -2860,7 +2797,7 @@
       <c r="F40" s="5"/>
       <c r="G40" s="9"/>
       <c r="H40" s="93" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="I40" s="59"/>
       <c r="J40" s="49"/>
@@ -2869,24 +2806,24 @@
       <c r="M40" s="52"/>
       <c r="N40" s="9"/>
       <c r="O40" s="14"/>
-      <c r="P40" s="8"/>
+      <c r="P40" s="57"/>
       <c r="Q40" s="16"/>
     </row>
-    <row r="41" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B41" s="51" t="s">
         <v>13</v>
       </c>
       <c r="C41" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="D41" s="121" t="s">
+      <c r="D41" s="115" t="s">
         <v>15</v>
       </c>
-      <c r="E41" s="109"/>
-      <c r="F41" s="113"/>
+      <c r="E41" s="116"/>
+      <c r="F41" s="117"/>
       <c r="G41" s="9"/>
       <c r="H41" s="94" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="I41" s="97"/>
       <c r="J41" s="84"/>
@@ -2895,18 +2832,18 @@
       <c r="M41" s="85"/>
       <c r="N41" s="9"/>
       <c r="O41" s="14"/>
-      <c r="P41" s="8"/>
+      <c r="P41" s="57"/>
       <c r="Q41" s="16"/>
     </row>
-    <row r="42" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B42" s="41"/>
       <c r="C42" s="41"/>
-      <c r="D42" s="110"/>
-      <c r="E42" s="116"/>
-      <c r="F42" s="117"/>
+      <c r="D42" s="108"/>
+      <c r="E42" s="109"/>
+      <c r="F42" s="110"/>
       <c r="G42" s="9"/>
       <c r="H42" s="94" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="I42" s="46"/>
       <c r="J42" s="42"/>
@@ -2915,40 +2852,40 @@
       <c r="M42" s="48"/>
       <c r="N42" s="9"/>
       <c r="O42" s="14"/>
-      <c r="P42" s="8"/>
+      <c r="P42" s="57"/>
       <c r="Q42" s="16"/>
     </row>
-    <row r="43" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="138"/>
+    <row r="43" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B43" s="41"/>
       <c r="C43" s="88"/>
-      <c r="D43" s="110"/>
-      <c r="E43" s="116"/>
-      <c r="F43" s="117"/>
+      <c r="D43" s="108"/>
+      <c r="E43" s="109"/>
+      <c r="F43" s="110"/>
       <c r="G43" s="9"/>
       <c r="H43" s="95" t="s">
-        <v>93</v>
-      </c>
-      <c r="I43" s="122" t="s">
-        <v>77</v>
-      </c>
-      <c r="J43" s="123"/>
-      <c r="K43" s="123"/>
-      <c r="L43" s="123"/>
-      <c r="M43" s="124"/>
+        <v>88</v>
+      </c>
+      <c r="I43" s="101" t="s">
+        <v>72</v>
+      </c>
+      <c r="J43" s="102"/>
+      <c r="K43" s="102"/>
+      <c r="L43" s="102"/>
+      <c r="M43" s="103"/>
       <c r="N43" s="9"/>
       <c r="O43" s="14"/>
-      <c r="P43" s="8"/>
+      <c r="P43" s="57"/>
       <c r="Q43" s="16"/>
     </row>
-    <row r="44" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B44" s="41"/>
       <c r="C44" s="88"/>
-      <c r="D44" s="110"/>
-      <c r="E44" s="116"/>
-      <c r="F44" s="117"/>
+      <c r="D44" s="108"/>
+      <c r="E44" s="109"/>
+      <c r="F44" s="110"/>
       <c r="G44" s="9"/>
       <c r="H44" s="94" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="I44" s="46" t="s">
         <v>51</v>
@@ -2967,18 +2904,18 @@
       </c>
       <c r="N44" s="9"/>
       <c r="O44" s="13"/>
-      <c r="P44" s="5"/>
+      <c r="P44" s="57"/>
       <c r="Q44" s="12"/>
     </row>
-    <row r="45" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B45" s="41"/>
       <c r="C45" s="41"/>
-      <c r="D45" s="110"/>
-      <c r="E45" s="116"/>
-      <c r="F45" s="117"/>
+      <c r="D45" s="108"/>
+      <c r="E45" s="109"/>
+      <c r="F45" s="110"/>
       <c r="G45" s="9"/>
       <c r="H45" s="94" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="I45" s="46"/>
       <c r="J45" s="42"/>
@@ -2990,37 +2927,37 @@
       <c r="P45" s="9"/>
       <c r="Q45" s="9"/>
     </row>
-    <row r="46" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B46" s="41"/>
       <c r="C46" s="41"/>
-      <c r="D46" s="110"/>
-      <c r="E46" s="116"/>
-      <c r="F46" s="117"/>
+      <c r="D46" s="108"/>
+      <c r="E46" s="109"/>
+      <c r="F46" s="110"/>
       <c r="G46" s="9"/>
       <c r="H46" s="95" t="s">
-        <v>95</v>
-      </c>
-      <c r="I46" s="122" t="s">
-        <v>78</v>
-      </c>
-      <c r="J46" s="123"/>
-      <c r="K46" s="123"/>
-      <c r="L46" s="123"/>
-      <c r="M46" s="124"/>
+        <v>90</v>
+      </c>
+      <c r="I46" s="101" t="s">
+        <v>73</v>
+      </c>
+      <c r="J46" s="102"/>
+      <c r="K46" s="102"/>
+      <c r="L46" s="102"/>
+      <c r="M46" s="103"/>
       <c r="N46" s="9"/>
       <c r="O46" s="9"/>
       <c r="P46" s="9"/>
       <c r="Q46" s="9"/>
     </row>
-    <row r="47" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B47" s="41"/>
       <c r="C47" s="41"/>
-      <c r="D47" s="110"/>
-      <c r="E47" s="116"/>
-      <c r="F47" s="117"/>
+      <c r="D47" s="108"/>
+      <c r="E47" s="109"/>
+      <c r="F47" s="110"/>
       <c r="G47" s="9"/>
       <c r="H47" s="94" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="I47" s="46"/>
       <c r="J47" s="42"/>
@@ -3029,12 +2966,12 @@
       <c r="M47" s="48"/>
       <c r="N47" s="9"/>
       <c r="O47" s="9" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="P47" s="9"/>
       <c r="Q47" s="9"/>
     </row>
-    <row r="48" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B48" s="28" t="s">
         <v>4</v>
       </c>
@@ -3047,7 +2984,7 @@
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
       <c r="H48" s="94" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I48" s="46"/>
       <c r="J48" s="42"/>
@@ -3059,7 +2996,7 @@
       <c r="P48" s="9"/>
       <c r="Q48" s="9"/>
     </row>
-    <row r="49" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B49" s="28" t="s">
         <v>5</v>
       </c>
@@ -3072,7 +3009,7 @@
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
       <c r="H49" s="94" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="I49" s="98"/>
       <c r="J49" s="86"/>
@@ -3084,7 +3021,7 @@
       <c r="P49" s="64"/>
       <c r="Q49" s="42"/>
     </row>
-    <row r="50" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B50" s="28"/>
       <c r="C50" s="43"/>
       <c r="D50" s="9"/>
@@ -3092,7 +3029,7 @@
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
       <c r="H50" s="96" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="I50" s="79"/>
       <c r="J50" s="80"/>
@@ -3110,7 +3047,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B51" s="28"/>
       <c r="C51" s="43"/>
       <c r="D51" s="9"/>
@@ -3128,7 +3065,7 @@
       <c r="P51" s="9"/>
       <c r="Q51" s="9"/>
     </row>
-    <row r="52" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B52" s="9"/>
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
@@ -3146,56 +3083,56 @@
       <c r="P52" s="9"/>
       <c r="Q52" s="9"/>
     </row>
-    <row r="53" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B53" s="115"/>
-      <c r="C53" s="115"/>
-      <c r="D53" s="115"/>
-      <c r="E53" s="115" t="s">
-        <v>64</v>
-      </c>
-      <c r="F53" s="115"/>
-      <c r="G53" s="115"/>
-      <c r="H53" s="115"/>
-      <c r="I53" s="115" t="s">
-        <v>74</v>
-      </c>
-      <c r="J53" s="115"/>
-      <c r="K53" s="115"/>
-      <c r="L53" s="115"/>
-      <c r="O53" s="114" t="s">
-        <v>98</v>
-      </c>
-      <c r="P53" s="114"/>
-      <c r="Q53" s="114"/>
-    </row>
-    <row r="54" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B54" s="115" t="s">
-        <v>65</v>
-      </c>
-      <c r="C54" s="115"/>
-      <c r="D54" s="115"/>
-      <c r="E54" s="114" t="s">
-        <v>80</v>
-      </c>
-      <c r="F54" s="114"/>
-      <c r="G54" s="114"/>
-      <c r="H54" s="114"/>
-      <c r="I54" s="115" t="s">
+    <row r="53" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="B53" s="111"/>
+      <c r="C53" s="111"/>
+      <c r="D53" s="111"/>
+      <c r="E53" s="111" t="s">
+        <v>59</v>
+      </c>
+      <c r="F53" s="111"/>
+      <c r="G53" s="111"/>
+      <c r="H53" s="111"/>
+      <c r="I53" s="111" t="s">
+        <v>69</v>
+      </c>
+      <c r="J53" s="111"/>
+      <c r="K53" s="111"/>
+      <c r="L53" s="111"/>
+      <c r="O53" s="126" t="s">
+        <v>93</v>
+      </c>
+      <c r="P53" s="126"/>
+      <c r="Q53" s="126"/>
+    </row>
+    <row r="54" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="B54" s="111" t="s">
+        <v>60</v>
+      </c>
+      <c r="C54" s="111"/>
+      <c r="D54" s="111"/>
+      <c r="E54" s="126" t="s">
         <v>75</v>
       </c>
-      <c r="J54" s="115"/>
-      <c r="K54" s="115"/>
-      <c r="L54" s="115"/>
+      <c r="F54" s="126"/>
+      <c r="G54" s="126"/>
+      <c r="H54" s="126"/>
+      <c r="I54" s="111" t="s">
+        <v>70</v>
+      </c>
+      <c r="J54" s="111"/>
+      <c r="K54" s="111"/>
+      <c r="L54" s="111"/>
       <c r="N54" t="s">
-        <v>66</v>
-      </c>
-      <c r="O54" s="115" t="s">
-        <v>76</v>
-      </c>
-      <c r="P54" s="115"/>
-      <c r="Q54" s="115"/>
-    </row>
-    <row r="55" spans="2:18" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+      <c r="O54" s="111" t="s">
+        <v>71</v>
+      </c>
+      <c r="P54" s="111"/>
+      <c r="Q54" s="111"/>
+    </row>
+    <row r="55" spans="2:18" ht="54.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B55" s="9"/>
       <c r="C55" s="9"/>
       <c r="D55" s="9"/>
@@ -3203,44 +3140,26 @@
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
       <c r="H55" s="9"/>
-      <c r="I55" s="101" t="s">
-        <v>81</v>
-      </c>
-      <c r="J55" s="101"/>
-      <c r="K55" s="101"/>
-      <c r="L55" s="101"/>
+      <c r="I55" s="118" t="s">
+        <v>76</v>
+      </c>
+      <c r="J55" s="118"/>
+      <c r="K55" s="118"/>
+      <c r="L55" s="118"/>
       <c r="M55" s="78"/>
       <c r="N55" s="9"/>
-      <c r="O55" s="101" t="s">
-        <v>82</v>
-      </c>
-      <c r="P55" s="101"/>
-      <c r="Q55" s="101"/>
+      <c r="O55" s="118" t="s">
+        <v>77</v>
+      </c>
+      <c r="P55" s="118"/>
+      <c r="Q55" s="118"/>
       <c r="R55" s="78"/>
     </row>
-    <row r="58" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:18" x14ac:dyDescent="0.35">
       <c r="E58" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="I31:M31"/>
-    <mergeCell ref="I34:M34"/>
-    <mergeCell ref="I43:M43"/>
-    <mergeCell ref="I46:M46"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D42:F42"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="O54:Q54"/>
-    <mergeCell ref="D44:F44"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D43:F43"/>
-    <mergeCell ref="D41:F41"/>
-    <mergeCell ref="D46:F46"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="D47:F47"/>
     <mergeCell ref="O55:Q55"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="D31:E31"/>
@@ -3257,6 +3176,24 @@
     <mergeCell ref="I54:L54"/>
     <mergeCell ref="I55:L55"/>
     <mergeCell ref="D45:F45"/>
+    <mergeCell ref="O54:Q54"/>
+    <mergeCell ref="D44:F44"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D43:F43"/>
+    <mergeCell ref="D41:F41"/>
+    <mergeCell ref="D46:F46"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="I31:M31"/>
+    <mergeCell ref="I34:M34"/>
+    <mergeCell ref="I43:M43"/>
+    <mergeCell ref="I46:M46"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="D32:E32"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.11811023622047245" right="0" top="0.39370078740157483" bottom="0" header="0" footer="0"/>
@@ -3269,7 +3206,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9D6F89B-2F67-41D8-AAA8-9E96940477A2}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
@@ -3280,7 +3217,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E74AD6C-8D0B-4421-9E6A-635D6611049A}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>

</xml_diff>

<commit_message>
chore: update teacher schedule template [v1.633]
</commit_message>
<xml_diff>
--- a/Template_Horario_Maestro.xlsx
+++ b/Template_Horario_Maestro.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\Customers\CBTis73\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rmartin\Downloads\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D0B559-8E3B-4744-99BD-CDF73E6461DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65A912CF-2C51-40A1-B55D-F5D850A96D31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="23596" windowHeight="15076" xr2:uid="{1066DCBB-7658-485D-B378-A5A8C35F949C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1066DCBB-7658-485D-B378-A5A8C35F949C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="99">
   <si>
     <t>Horas</t>
   </si>
@@ -191,15 +191,24 @@
     <t>DOCENTES</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Asignatura</t>
   </si>
   <si>
     <t>CLAVE</t>
   </si>
   <si>
+    <t>LUNES</t>
+  </si>
+  <si>
+    <t>MARTES</t>
+  </si>
+  <si>
+    <t>JUEVES</t>
+  </si>
+  <si>
+    <t>VIERNES</t>
+  </si>
+  <si>
     <t>HORARIO TURNO VESPERTINO</t>
   </si>
   <si>
@@ -215,6 +224,9 @@
     <t>la DGETI</t>
   </si>
   <si>
+    <t>MIERC.</t>
+  </si>
+  <si>
     <t>Yolanda Morales Miranda</t>
   </si>
   <si>
@@ -264,12 +276,6 @@
   </si>
   <si>
     <t>Jefe de Depto. de Servicios Docentes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Firma en ausencia y suplencia del Subirector del Cbtis No. 73 El  C. Jorge Omar Hernández Doria, con fundamento en el artículo 54 del Reglamento Interior de la SEP, en ejercicio de las Funciones asignadas en el Oficio 220(1)5419/2020.			</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Firma en ausencia y suplencia del Director del Cbtis No. 73 El  C. José Oliverio Márquez  Muñoz, con fundamento en el artículo 54 del Reglamento Interior de la SEP, en ejercicio de las Funciones asignadas en el Oficio 220(1)5419/2020.			</t>
   </si>
   <si>
     <t>7:00-7:50</t>
@@ -406,7 +412,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="59">
+  <borders count="58">
     <border>
       <left/>
       <right/>
@@ -455,17 +461,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -1154,7 +1149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1177,68 +1172,70 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1251,218 +1248,209 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="20" fontId="2" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1913,100 +1901,100 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58F58D38-BD95-48DF-854F-C3512D201DF1}">
   <dimension ref="A4:AT58"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.73046875" defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.3984375" customWidth="1"/>
-    <col min="2" max="2" width="9.73046875" customWidth="1"/>
-    <col min="3" max="3" width="12.3984375" customWidth="1"/>
-    <col min="5" max="5" width="37.1328125" customWidth="1"/>
-    <col min="6" max="6" width="6.265625" customWidth="1"/>
-    <col min="7" max="7" width="4.3984375" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="13" width="8.86328125" customWidth="1"/>
-    <col min="14" max="14" width="6.73046875" customWidth="1"/>
-    <col min="15" max="17" width="9.73046875" customWidth="1"/>
-    <col min="18" max="18" width="9.3984375" customWidth="1"/>
+    <col min="1" max="1" width="4.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="37.140625" customWidth="1"/>
+    <col min="6" max="6" width="6.28515625" customWidth="1"/>
+    <col min="7" max="7" width="4.42578125" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" customWidth="1"/>
+    <col min="9" max="13" width="8.85546875" customWidth="1"/>
+    <col min="14" max="14" width="6.7109375" customWidth="1"/>
+    <col min="15" max="17" width="9.7109375" customWidth="1"/>
+    <col min="18" max="18" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:46" ht="15" x14ac:dyDescent="0.35">
-      <c r="B4" s="56" t="s">
-        <v>57</v>
-      </c>
-      <c r="C4" s="56"/>
-      <c r="D4" s="56"/>
-      <c r="E4" s="56"/>
-      <c r="F4" s="56"/>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
-      <c r="I4" s="56"/>
-      <c r="J4" s="56"/>
-      <c r="K4" s="56"/>
-      <c r="L4" s="56"/>
-      <c r="M4" s="56"/>
-      <c r="N4" s="56"/>
-      <c r="O4" s="56"/>
-      <c r="P4" s="56"/>
-      <c r="Q4" s="56"/>
-    </row>
-    <row r="5" spans="1:46" ht="15" x14ac:dyDescent="0.35">
-      <c r="B5" s="56" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" s="56"/>
-      <c r="D5" s="56"/>
-      <c r="E5" s="56"/>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
-      <c r="H5" s="56"/>
-      <c r="I5" s="56"/>
-      <c r="J5" s="56"/>
-      <c r="K5" s="56"/>
-      <c r="L5" s="56"/>
-      <c r="M5" s="56"/>
-      <c r="N5" s="56"/>
-      <c r="O5" s="56"/>
-      <c r="P5" s="56"/>
-      <c r="Q5" s="56"/>
-    </row>
-    <row r="6" spans="1:46" ht="15" x14ac:dyDescent="0.35">
-      <c r="B6" s="56" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" s="56"/>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="56"/>
-      <c r="I6" s="56"/>
-      <c r="J6" s="56"/>
-      <c r="K6" s="56"/>
-      <c r="L6" s="56"/>
-      <c r="M6" s="56"/>
-      <c r="N6" s="56"/>
-      <c r="O6" s="56"/>
-      <c r="P6" s="56"/>
-      <c r="Q6" s="56"/>
-    </row>
-    <row r="7" spans="1:46" ht="15" x14ac:dyDescent="0.35">
-      <c r="B7" s="56"/>
-      <c r="C7" s="56"/>
-      <c r="D7" s="56"/>
-      <c r="E7" s="56"/>
-      <c r="F7" s="56"/>
-      <c r="G7" s="56"/>
-      <c r="H7" s="56"/>
-      <c r="I7" s="56"/>
-      <c r="J7" s="56"/>
-      <c r="K7" s="56"/>
-      <c r="L7" s="56"/>
-      <c r="M7" s="56"/>
-      <c r="N7" s="56"/>
-      <c r="O7" s="56"/>
-      <c r="P7" s="56"/>
-      <c r="Q7" s="56"/>
-    </row>
-    <row r="8" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:46" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="B4" s="55" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="55"/>
+      <c r="L4" s="55"/>
+      <c r="M4" s="55"/>
+      <c r="N4" s="55"/>
+      <c r="O4" s="55"/>
+      <c r="P4" s="55"/>
+      <c r="Q4" s="55"/>
+    </row>
+    <row r="5" spans="1:46" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="B5" s="55" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="55"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="55"/>
+      <c r="H5" s="55"/>
+      <c r="I5" s="55"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="55"/>
+      <c r="L5" s="55"/>
+      <c r="M5" s="55"/>
+      <c r="N5" s="55"/>
+      <c r="O5" s="55"/>
+      <c r="P5" s="55"/>
+      <c r="Q5" s="55"/>
+    </row>
+    <row r="6" spans="1:46" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="B6" s="55" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
+      <c r="H6" s="55"/>
+      <c r="I6" s="55"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="55"/>
+      <c r="L6" s="55"/>
+      <c r="M6" s="55"/>
+      <c r="N6" s="55"/>
+      <c r="O6" s="55"/>
+      <c r="P6" s="55"/>
+      <c r="Q6" s="55"/>
+    </row>
+    <row r="7" spans="1:46" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="B7" s="55"/>
+      <c r="C7" s="55"/>
+      <c r="D7" s="55"/>
+      <c r="E7" s="55"/>
+      <c r="F7" s="55"/>
+      <c r="G7" s="55"/>
+      <c r="H7" s="55"/>
+      <c r="I7" s="55"/>
+      <c r="J7" s="55"/>
+      <c r="K7" s="55"/>
+      <c r="L7" s="55"/>
+      <c r="M7" s="55"/>
+      <c r="N7" s="55"/>
+      <c r="O7" s="55"/>
+      <c r="P7" s="55"/>
+      <c r="Q7" s="55"/>
+    </row>
+    <row r="8" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -2025,7 +2013,7 @@
       <c r="AB8" s="4"/>
       <c r="AC8" s="4"/>
     </row>
-    <row r="9" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
         <v>18</v>
       </c>
@@ -2055,7 +2043,7 @@
       </c>
       <c r="O9" s="8"/>
       <c r="P9" s="8"/>
-      <c r="Q9" s="10"/>
+      <c r="Q9" s="15"/>
       <c r="R9" s="4"/>
       <c r="S9" s="4"/>
       <c r="T9" s="4"/>
@@ -2069,8 +2057,8 @@
       <c r="AB9" s="4"/>
       <c r="AC9" s="4"/>
     </row>
-    <row r="10" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="11" t="s">
+    <row r="10" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="10" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="9"/>
@@ -2089,13 +2077,13 @@
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="9" t="s">
+      <c r="M10" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="O10" s="9"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
       <c r="P10" s="5"/>
-      <c r="Q10" s="12"/>
+      <c r="Q10" s="11"/>
       <c r="R10" s="4"/>
       <c r="S10" s="4"/>
       <c r="T10" s="4"/>
@@ -2126,8 +2114,8 @@
       <c r="AS10" s="4"/>
       <c r="AT10" s="4"/>
     </row>
-    <row r="11" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="13"/>
+    <row r="11" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="12"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
@@ -2142,10 +2130,10 @@
       <c r="N11" s="5"/>
       <c r="O11" s="5"/>
       <c r="P11" s="5"/>
-      <c r="Q11" s="12"/>
-    </row>
-    <row r="12" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="14" t="s">
+      <c r="Q11" s="11"/>
+    </row>
+    <row r="12" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="13" t="s">
         <v>24</v>
       </c>
       <c r="C12" s="8"/>
@@ -2155,7 +2143,7 @@
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
-      <c r="J12" s="15" t="s">
+      <c r="J12" s="14" t="s">
         <v>25</v>
       </c>
       <c r="K12" s="8"/>
@@ -2164,35 +2152,35 @@
       <c r="N12" s="8"/>
       <c r="O12" s="8"/>
       <c r="P12" s="8"/>
-      <c r="Q12" s="16"/>
-    </row>
-    <row r="13" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="14" t="s">
+      <c r="Q12" s="15"/>
+    </row>
+    <row r="13" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
-      <c r="G13" s="15" t="s">
-        <v>95</v>
+      <c r="G13" s="14" t="s">
+        <v>97</v>
       </c>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
-      <c r="K13" s="15" t="s">
-        <v>94</v>
+      <c r="K13" s="14" t="s">
+        <v>96</v>
       </c>
       <c r="L13" s="8"/>
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
       <c r="O13" s="8"/>
       <c r="P13" s="8"/>
-      <c r="Q13" s="16"/>
-    </row>
-    <row r="14" spans="1:46" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="Q13" s="15"/>
+    </row>
+    <row r="14" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="13" t="s">
         <v>27</v>
       </c>
       <c r="C14" s="8"/>
@@ -2202,224 +2190,224 @@
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
-      <c r="H14" s="15" t="s">
-        <v>96</v>
+      <c r="H14" s="14" t="s">
+        <v>98</v>
       </c>
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
       <c r="K14" s="8"/>
-      <c r="L14" s="15"/>
+      <c r="L14" s="14"/>
       <c r="M14" s="8"/>
-      <c r="N14" s="15"/>
+      <c r="N14" s="14"/>
       <c r="O14" s="8"/>
       <c r="P14" s="8"/>
-      <c r="Q14" s="16"/>
-    </row>
-    <row r="15" spans="1:46" x14ac:dyDescent="0.35">
-      <c r="B15" s="17" t="s">
+      <c r="Q14" s="15"/>
+    </row>
+    <row r="15" spans="1:46" x14ac:dyDescent="0.2">
+      <c r="B15" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="20"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="19"/>
       <c r="F15" s="7"/>
       <c r="G15" s="7"/>
       <c r="H15" s="9"/>
       <c r="I15" s="7"/>
-      <c r="J15" s="21" t="s">
+      <c r="J15" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="K15" s="22"/>
-      <c r="L15" s="23"/>
+      <c r="K15" s="21"/>
+      <c r="L15" s="22"/>
       <c r="M15" s="9"/>
       <c r="N15" s="9"/>
       <c r="O15" s="9"/>
       <c r="P15" s="9"/>
-      <c r="Q15" s="24"/>
-    </row>
-    <row r="16" spans="1:46" x14ac:dyDescent="0.35">
-      <c r="B16" s="25" t="s">
+      <c r="Q15" s="23"/>
+    </row>
+    <row r="16" spans="1:46" x14ac:dyDescent="0.2">
+      <c r="B16" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="26" t="s">
+      <c r="D16" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="E16" s="23"/>
+      <c r="E16" s="22"/>
       <c r="F16" s="9"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
       <c r="I16" s="9"/>
-      <c r="J16" s="27" t="s">
+      <c r="J16" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="K16" s="28"/>
-      <c r="L16" s="119" t="s">
+      <c r="K16" s="27"/>
+      <c r="L16" s="116" t="s">
         <v>49</v>
       </c>
-      <c r="M16" s="120"/>
-      <c r="N16" s="120"/>
-      <c r="O16" s="120"/>
-      <c r="P16" s="120"/>
-      <c r="Q16" s="121"/>
-    </row>
-    <row r="17" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="25" t="s">
+      <c r="M16" s="117"/>
+      <c r="N16" s="117"/>
+      <c r="O16" s="117"/>
+      <c r="P16" s="117"/>
+      <c r="Q16" s="118"/>
+    </row>
+    <row r="17" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C17" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="29" t="s">
+      <c r="D17" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="23"/>
+      <c r="E17" s="22"/>
       <c r="F17" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="G17" s="30"/>
-      <c r="H17" s="28" t="s">
+      <c r="G17" s="29"/>
+      <c r="H17" s="27" t="s">
         <v>40</v>
       </c>
       <c r="I17" s="9"/>
-      <c r="J17" s="23" t="s">
+      <c r="J17" s="22" t="s">
         <v>41</v>
       </c>
       <c r="K17" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="L17" s="31"/>
+      <c r="L17" s="30"/>
       <c r="M17" s="5"/>
       <c r="N17" s="5"/>
       <c r="O17" s="5"/>
       <c r="P17" s="5"/>
-      <c r="Q17" s="12"/>
-    </row>
-    <row r="18" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="32" t="s">
+      <c r="Q17" s="11"/>
+    </row>
+    <row r="18" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="55" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="26" t="s">
+      <c r="C18" s="54" t="s">
+        <v>61</v>
+      </c>
+      <c r="D18" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="E18" s="31"/>
+      <c r="E18" s="30"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="33"/>
+      <c r="G18" s="32"/>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
-      <c r="J18" s="31" t="s">
+      <c r="J18" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="K18" s="34"/>
-      <c r="L18" s="31"/>
+      <c r="K18" s="33"/>
+      <c r="L18" s="30"/>
       <c r="M18" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="N18" s="35"/>
+      <c r="N18" s="34"/>
       <c r="O18" s="8"/>
       <c r="P18" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="Q18" s="16"/>
+      <c r="Q18" s="15"/>
       <c r="S18" s="3"/>
     </row>
-    <row r="19" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="44"/>
-      <c r="C19" s="45"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="66"/>
+    <row r="19" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="43"/>
+      <c r="C19" s="44"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="65"/>
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
-      <c r="J19" s="108"/>
-      <c r="K19" s="124"/>
-      <c r="L19" s="15"/>
-      <c r="M19" s="60"/>
-      <c r="N19" s="54"/>
-      <c r="O19" s="40"/>
-      <c r="P19" s="60"/>
-      <c r="Q19" s="16"/>
-    </row>
-    <row r="20" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B20" s="36"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="15"/>
+      <c r="J19" s="107"/>
+      <c r="K19" s="121"/>
+      <c r="L19" s="14"/>
+      <c r="M19" s="59"/>
+      <c r="N19" s="53"/>
+      <c r="O19" s="39"/>
+      <c r="P19" s="59"/>
+      <c r="Q19" s="15"/>
+    </row>
+    <row r="20" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="35"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="14"/>
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="35"/>
-      <c r="L20" s="15"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="34"/>
+      <c r="L20" s="14"/>
       <c r="M20" s="8"/>
-      <c r="N20" s="35"/>
+      <c r="N20" s="34"/>
       <c r="O20" s="8"/>
       <c r="P20" s="8"/>
-      <c r="Q20" s="16"/>
-    </row>
-    <row r="21" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B21" s="36"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="15"/>
+      <c r="Q20" s="15"/>
+    </row>
+    <row r="21" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="35"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="14"/>
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="I21" s="8"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="35"/>
-      <c r="L21" s="15"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="34"/>
+      <c r="L21" s="14"/>
       <c r="M21" s="8"/>
-      <c r="N21" s="35"/>
+      <c r="N21" s="34"/>
       <c r="O21" s="8"/>
       <c r="P21" s="8"/>
-      <c r="Q21" s="16"/>
-    </row>
-    <row r="22" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B22" s="36"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="15"/>
+      <c r="Q21" s="15"/>
+    </row>
+    <row r="22" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="35"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="14"/>
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
       <c r="I22" s="8"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="35"/>
-      <c r="L22" s="15"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="34"/>
+      <c r="L22" s="14"/>
       <c r="M22" s="8"/>
-      <c r="N22" s="35"/>
+      <c r="N22" s="34"/>
       <c r="O22" s="8"/>
       <c r="P22" s="8"/>
-      <c r="Q22" s="16"/>
-    </row>
-    <row r="23" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B23" s="38"/>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="31"/>
+      <c r="Q22" s="15"/>
+    </row>
+    <row r="23" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="37"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="30"/>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
       <c r="H23" s="8"/>
       <c r="I23" s="8"/>
-      <c r="J23" s="31"/>
-      <c r="K23" s="34"/>
-      <c r="L23" s="31"/>
+      <c r="J23" s="30"/>
+      <c r="K23" s="33"/>
+      <c r="L23" s="30"/>
       <c r="M23" s="5"/>
-      <c r="N23" s="34"/>
+      <c r="N23" s="33"/>
       <c r="O23" s="5"/>
       <c r="P23" s="5"/>
-      <c r="Q23" s="12"/>
-      <c r="R23" s="53"/>
-    </row>
-    <row r="24" spans="2:23" x14ac:dyDescent="0.35">
+      <c r="Q23" s="11"/>
+      <c r="R23" s="52"/>
+    </row>
+    <row r="24" spans="2:23" x14ac:dyDescent="0.2">
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
@@ -2436,10 +2424,10 @@
       <c r="O24" s="9"/>
       <c r="P24" s="9"/>
       <c r="Q24" s="9"/>
-      <c r="R24" s="53"/>
+      <c r="R24" s="52"/>
       <c r="W24" s="2"/>
     </row>
-    <row r="25" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B25" s="9" t="s">
         <v>16</v>
       </c>
@@ -2458,275 +2446,277 @@
       <c r="O25" s="9"/>
       <c r="P25" s="9"/>
       <c r="Q25" s="9"/>
-      <c r="R25" s="53"/>
-    </row>
-    <row r="26" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R25" s="52"/>
+    </row>
+    <row r="26" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
-      <c r="H26" s="125" t="s">
+      <c r="H26" s="122" t="s">
         <v>11</v>
       </c>
-      <c r="I26" s="116"/>
-      <c r="J26" s="116"/>
-      <c r="K26" s="116"/>
-      <c r="L26" s="116"/>
-      <c r="M26" s="117"/>
+      <c r="I26" s="113"/>
+      <c r="J26" s="113"/>
+      <c r="K26" s="113"/>
+      <c r="L26" s="113"/>
+      <c r="M26" s="114"/>
       <c r="N26" s="9"/>
-      <c r="O26" s="71"/>
-      <c r="P26" s="40" t="s">
+      <c r="O26" s="70"/>
+      <c r="P26" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="Q26" s="72"/>
-      <c r="R26" s="53"/>
-    </row>
-    <row r="27" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B27" s="73" t="s">
+      <c r="Q26" s="71"/>
+      <c r="R26" s="52"/>
+    </row>
+    <row r="27" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="72" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="74" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="113" t="s">
+        <v>51</v>
+      </c>
+      <c r="E27" s="113"/>
+      <c r="F27" s="74" t="s">
+        <v>36</v>
+      </c>
+      <c r="G27" s="9"/>
+      <c r="H27" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="I27" s="98" t="s">
+        <v>6</v>
+      </c>
+      <c r="J27" s="50" t="s">
+        <v>7</v>
+      </c>
+      <c r="K27" s="50" t="s">
+        <v>8</v>
+      </c>
+      <c r="L27" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="M27" s="99" t="s">
+        <v>10</v>
+      </c>
+      <c r="N27" s="9"/>
+      <c r="O27" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="C27" s="75" t="s">
-        <v>14</v>
-      </c>
-      <c r="D27" s="116" t="s">
-        <v>52</v>
-      </c>
-      <c r="E27" s="116"/>
-      <c r="F27" s="75" t="s">
-        <v>36</v>
-      </c>
-      <c r="G27" s="9"/>
-      <c r="H27" s="50" t="s">
-        <v>0</v>
-      </c>
-      <c r="I27" s="99" t="s">
-        <v>6</v>
-      </c>
-      <c r="J27" s="51" t="s">
-        <v>7</v>
-      </c>
-      <c r="K27" s="51" t="s">
-        <v>8</v>
-      </c>
-      <c r="L27" s="51" t="s">
-        <v>9</v>
-      </c>
-      <c r="M27" s="100" t="s">
-        <v>10</v>
-      </c>
-      <c r="N27" s="9"/>
-      <c r="O27" s="14"/>
-      <c r="P27" s="57"/>
-      <c r="Q27" s="58"/>
-      <c r="R27" s="53"/>
-    </row>
-    <row r="28" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B28" s="67"/>
-      <c r="C28" s="68"/>
-      <c r="D28" s="122"/>
-      <c r="E28" s="123"/>
-      <c r="F28" s="74"/>
+      <c r="P27" s="56"/>
+      <c r="Q27" s="57"/>
+      <c r="R27" s="52"/>
+    </row>
+    <row r="28" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="66"/>
+      <c r="C28" s="67"/>
+      <c r="D28" s="119"/>
+      <c r="E28" s="120"/>
+      <c r="F28" s="73"/>
       <c r="G28" s="9"/>
-      <c r="H28" s="89" t="s">
-        <v>78</v>
-      </c>
-      <c r="I28" s="97"/>
-      <c r="J28" s="84"/>
-      <c r="K28" s="49"/>
-      <c r="L28" s="84"/>
-      <c r="M28" s="85"/>
+      <c r="H28" s="88" t="s">
+        <v>80</v>
+      </c>
+      <c r="I28" s="96"/>
+      <c r="J28" s="83"/>
+      <c r="K28" s="48"/>
+      <c r="L28" s="83"/>
+      <c r="M28" s="84"/>
       <c r="N28" s="9"/>
-      <c r="O28" s="14"/>
-      <c r="P28" s="57"/>
-      <c r="Q28" s="58"/>
-      <c r="R28" s="53"/>
-    </row>
-    <row r="29" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B29" s="67"/>
-      <c r="C29" s="74"/>
-      <c r="D29" s="104"/>
-      <c r="E29" s="105"/>
-      <c r="F29" s="74"/>
+      <c r="O28" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="P28" s="56"/>
+      <c r="Q28" s="57"/>
+      <c r="R28" s="52"/>
+    </row>
+    <row r="29" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="66"/>
+      <c r="C29" s="73"/>
+      <c r="D29" s="103"/>
+      <c r="E29" s="104"/>
+      <c r="F29" s="73"/>
       <c r="G29" s="9"/>
-      <c r="H29" s="90" t="s">
-        <v>79</v>
-      </c>
-      <c r="I29" s="46"/>
-      <c r="J29" s="42"/>
-      <c r="K29" s="84"/>
-      <c r="L29" s="42"/>
-      <c r="M29" s="48"/>
+      <c r="H29" s="89" t="s">
+        <v>81</v>
+      </c>
+      <c r="I29" s="45"/>
+      <c r="J29" s="41"/>
+      <c r="K29" s="83"/>
+      <c r="L29" s="41"/>
+      <c r="M29" s="47"/>
       <c r="N29" s="9"/>
-      <c r="O29" s="14"/>
-      <c r="P29" s="57"/>
-      <c r="Q29" s="58"/>
-      <c r="R29" s="53"/>
-    </row>
-    <row r="30" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="67"/>
-      <c r="C30" s="74"/>
-      <c r="D30" s="104"/>
-      <c r="E30" s="105"/>
-      <c r="F30" s="74"/>
+      <c r="O29" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="P29" s="56"/>
+      <c r="Q29" s="57"/>
+      <c r="R29" s="52"/>
+    </row>
+    <row r="30" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="66"/>
+      <c r="C30" s="73"/>
+      <c r="D30" s="103"/>
+      <c r="E30" s="104"/>
+      <c r="F30" s="73"/>
       <c r="G30" s="9"/>
-      <c r="H30" s="90" t="s">
-        <v>80</v>
-      </c>
-      <c r="I30" s="46"/>
-      <c r="J30" s="42"/>
-      <c r="K30" s="42"/>
-      <c r="L30" s="42"/>
-      <c r="M30" s="48"/>
+      <c r="H30" s="89" t="s">
+        <v>82</v>
+      </c>
+      <c r="I30" s="45"/>
+      <c r="J30" s="41"/>
+      <c r="K30" s="41"/>
+      <c r="L30" s="41"/>
+      <c r="M30" s="47"/>
       <c r="N30" s="9"/>
-      <c r="O30" s="14"/>
-      <c r="P30" s="57"/>
-      <c r="Q30" s="58"/>
-      <c r="R30" s="53"/>
-    </row>
-    <row r="31" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B31" s="47"/>
-      <c r="C31" s="70"/>
-      <c r="D31" s="104"/>
-      <c r="E31" s="105"/>
-      <c r="F31" s="69"/>
+      <c r="O30" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="P30" s="56"/>
+      <c r="Q30" s="57"/>
+      <c r="R30" s="52"/>
+    </row>
+    <row r="31" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="46"/>
+      <c r="C31" s="69"/>
+      <c r="D31" s="103"/>
+      <c r="E31" s="104"/>
+      <c r="F31" s="68"/>
       <c r="G31" s="9"/>
-      <c r="H31" s="91" t="s">
-        <v>81</v>
-      </c>
-      <c r="I31" s="101" t="s">
-        <v>72</v>
-      </c>
-      <c r="J31" s="102"/>
-      <c r="K31" s="102"/>
-      <c r="L31" s="102"/>
-      <c r="M31" s="103"/>
+      <c r="H31" s="90" t="s">
+        <v>83</v>
+      </c>
+      <c r="I31" s="100" t="s">
+        <v>76</v>
+      </c>
+      <c r="J31" s="101"/>
+      <c r="K31" s="101"/>
+      <c r="L31" s="101"/>
+      <c r="M31" s="102"/>
       <c r="N31" s="9"/>
-      <c r="O31" s="14"/>
-      <c r="P31" s="57"/>
-      <c r="Q31" s="58"/>
-      <c r="R31" s="53"/>
-    </row>
-    <row r="32" spans="2:23" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B32" s="47"/>
-      <c r="C32" s="70"/>
-      <c r="D32" s="104"/>
-      <c r="E32" s="105"/>
-      <c r="F32" s="70"/>
+      <c r="O31" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="P31" s="56"/>
+      <c r="Q31" s="57"/>
+      <c r="R31" s="52"/>
+    </row>
+    <row r="32" spans="2:23" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="46"/>
+      <c r="C32" s="69"/>
+      <c r="D32" s="103"/>
+      <c r="E32" s="104"/>
+      <c r="F32" s="69"/>
       <c r="G32" s="9"/>
-      <c r="H32" s="90" t="s">
-        <v>82</v>
-      </c>
-      <c r="I32" s="46"/>
-      <c r="J32" s="42"/>
-      <c r="K32" s="42"/>
-      <c r="L32" s="42"/>
-      <c r="M32" s="48"/>
+      <c r="H32" s="89" t="s">
+        <v>84</v>
+      </c>
+      <c r="I32" s="45"/>
+      <c r="J32" s="41"/>
+      <c r="K32" s="41"/>
+      <c r="L32" s="41"/>
+      <c r="M32" s="47"/>
       <c r="N32" s="9"/>
-      <c r="O32" s="14"/>
-      <c r="P32" s="57"/>
-      <c r="Q32" s="58"/>
-      <c r="R32" s="53"/>
-    </row>
-    <row r="33" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B33" s="47"/>
-      <c r="C33" s="70"/>
-      <c r="D33" s="104"/>
-      <c r="E33" s="105"/>
-      <c r="F33" s="70"/>
+      <c r="O32" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="P32" s="56"/>
+      <c r="Q32" s="57"/>
+      <c r="R32" s="52"/>
+    </row>
+    <row r="33" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="46"/>
+      <c r="C33" s="69"/>
+      <c r="D33" s="103"/>
+      <c r="E33" s="104"/>
+      <c r="F33" s="69"/>
       <c r="G33" s="9"/>
-      <c r="H33" s="90" t="s">
-        <v>83</v>
-      </c>
-      <c r="I33" s="46" t="s">
-        <v>51</v>
-      </c>
-      <c r="J33" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="K33" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="L33" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="M33" s="48" t="s">
-        <v>51</v>
-      </c>
+      <c r="H33" s="89" t="s">
+        <v>85</v>
+      </c>
+      <c r="I33" s="45"/>
+      <c r="J33" s="41"/>
+      <c r="K33" s="41"/>
+      <c r="L33" s="41"/>
+      <c r="M33" s="47"/>
       <c r="N33" s="9"/>
-      <c r="O33" s="14"/>
-      <c r="P33" s="57"/>
-      <c r="Q33" s="58"/>
-      <c r="R33" s="53"/>
-    </row>
-    <row r="34" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B34" s="47"/>
-      <c r="C34" s="70"/>
-      <c r="D34" s="112"/>
-      <c r="E34" s="113"/>
-      <c r="F34" s="62"/>
+      <c r="O33" s="13"/>
+      <c r="P33" s="56"/>
+      <c r="Q33" s="57"/>
+      <c r="R33" s="52"/>
+    </row>
+    <row r="34" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="46"/>
+      <c r="C34" s="69"/>
+      <c r="D34" s="109"/>
+      <c r="E34" s="110"/>
+      <c r="F34" s="61"/>
       <c r="G34" s="9"/>
-      <c r="H34" s="91" t="s">
-        <v>84</v>
-      </c>
-      <c r="I34" s="101" t="s">
-        <v>73</v>
-      </c>
-      <c r="J34" s="102"/>
-      <c r="K34" s="102"/>
-      <c r="L34" s="102"/>
-      <c r="M34" s="103"/>
+      <c r="H34" s="90" t="s">
+        <v>86</v>
+      </c>
+      <c r="I34" s="100" t="s">
+        <v>77</v>
+      </c>
+      <c r="J34" s="101"/>
+      <c r="K34" s="101"/>
+      <c r="L34" s="101"/>
+      <c r="M34" s="102"/>
       <c r="N34" s="9"/>
-      <c r="O34" s="13"/>
-      <c r="P34" s="57"/>
-      <c r="Q34" s="12"/>
-    </row>
-    <row r="35" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B35" s="47"/>
-      <c r="C35" s="70"/>
-      <c r="D35" s="114"/>
-      <c r="E35" s="105"/>
-      <c r="F35" s="70"/>
+      <c r="O34" s="12"/>
+      <c r="P34" s="8"/>
+      <c r="Q34" s="11"/>
+    </row>
+    <row r="35" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="46"/>
+      <c r="C35" s="69"/>
+      <c r="D35" s="111"/>
+      <c r="E35" s="104"/>
+      <c r="F35" s="69"/>
       <c r="G35" s="9"/>
-      <c r="H35" s="90" t="s">
-        <v>62</v>
-      </c>
-      <c r="I35" s="46"/>
-      <c r="J35" s="42"/>
-      <c r="K35" s="42"/>
-      <c r="L35" s="42"/>
-      <c r="M35" s="48"/>
+      <c r="H35" s="89" t="s">
+        <v>66</v>
+      </c>
+      <c r="I35" s="45"/>
+      <c r="J35" s="41"/>
+      <c r="K35" s="41"/>
+      <c r="L35" s="41"/>
+      <c r="M35" s="47"/>
       <c r="N35" s="9"/>
-      <c r="O35" s="13"/>
-      <c r="P35" s="57"/>
-      <c r="Q35" s="12"/>
-    </row>
-    <row r="36" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B36" s="76"/>
-      <c r="C36" s="77"/>
-      <c r="D36" s="106"/>
-      <c r="E36" s="107"/>
-      <c r="F36" s="63"/>
+      <c r="O35" s="12"/>
+      <c r="P35" s="8"/>
+      <c r="Q35" s="11"/>
+    </row>
+    <row r="36" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="75"/>
+      <c r="C36" s="76"/>
+      <c r="D36" s="105"/>
+      <c r="E36" s="106"/>
+      <c r="F36" s="62"/>
       <c r="G36" s="9"/>
-      <c r="H36" s="90" t="s">
-        <v>85</v>
-      </c>
-      <c r="I36" s="46"/>
-      <c r="J36" s="42"/>
-      <c r="K36" s="42"/>
-      <c r="L36" s="42"/>
-      <c r="M36" s="48"/>
+      <c r="H36" s="89" t="s">
+        <v>87</v>
+      </c>
+      <c r="I36" s="45"/>
+      <c r="J36" s="41"/>
+      <c r="K36" s="41"/>
+      <c r="L36" s="41"/>
+      <c r="M36" s="47"/>
       <c r="N36" s="9"/>
-      <c r="O36" s="14"/>
-      <c r="P36" s="57"/>
-      <c r="Q36" s="16"/>
-    </row>
-    <row r="37" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O36" s="13"/>
+      <c r="P36" s="8"/>
+      <c r="Q36" s="15"/>
+    </row>
+    <row r="37" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B37" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C37" s="61">
+      <c r="C37" s="60">
         <f>SUM(C28:C36)</f>
         <v>0</v>
       </c>
@@ -2734,40 +2724,40 @@
       <c r="E37" s="9"/>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
-      <c r="H37" s="90" t="s">
-        <v>86</v>
-      </c>
-      <c r="I37" s="46"/>
-      <c r="J37" s="42"/>
-      <c r="K37" s="42"/>
-      <c r="L37" s="42"/>
-      <c r="M37" s="48"/>
+      <c r="H37" s="89" t="s">
+        <v>88</v>
+      </c>
+      <c r="I37" s="45"/>
+      <c r="J37" s="41"/>
+      <c r="K37" s="41"/>
+      <c r="L37" s="41"/>
+      <c r="M37" s="47"/>
       <c r="N37" s="9"/>
-      <c r="O37" s="14"/>
-      <c r="P37" s="57"/>
-      <c r="Q37" s="16"/>
-    </row>
-    <row r="38" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O37" s="13"/>
+      <c r="P37" s="8"/>
+      <c r="Q37" s="15"/>
+    </row>
+    <row r="38" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
-      <c r="H38" s="89" t="s">
-        <v>87</v>
-      </c>
-      <c r="I38" s="79"/>
-      <c r="J38" s="80"/>
-      <c r="K38" s="80"/>
-      <c r="L38" s="80"/>
-      <c r="M38" s="81"/>
+      <c r="H38" s="88" t="s">
+        <v>89</v>
+      </c>
+      <c r="I38" s="78"/>
+      <c r="J38" s="79"/>
+      <c r="K38" s="79"/>
+      <c r="L38" s="79"/>
+      <c r="M38" s="80"/>
       <c r="N38" s="9"/>
-      <c r="O38" s="14"/>
-      <c r="P38" s="57"/>
-      <c r="Q38" s="16"/>
-    </row>
-    <row r="39" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O38" s="13"/>
+      <c r="P38" s="8"/>
+      <c r="Q38" s="15"/>
+    </row>
+    <row r="39" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B39" s="9" t="s">
         <v>17</v>
       </c>
@@ -2776,206 +2766,196 @@
       <c r="E39" s="9"/>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
-      <c r="H39" s="92"/>
-      <c r="I39" s="82" t="s">
-        <v>54</v>
-      </c>
-      <c r="J39" s="82"/>
-      <c r="K39" s="82"/>
-      <c r="L39" s="82"/>
-      <c r="M39" s="83"/>
+      <c r="H39" s="91"/>
+      <c r="I39" s="81" t="s">
+        <v>57</v>
+      </c>
+      <c r="J39" s="81"/>
+      <c r="K39" s="81"/>
+      <c r="L39" s="81"/>
+      <c r="M39" s="82"/>
       <c r="N39" s="9"/>
-      <c r="O39" s="14"/>
-      <c r="P39" s="57"/>
-      <c r="Q39" s="16"/>
-    </row>
-    <row r="40" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O39" s="13"/>
+      <c r="P39" s="8"/>
+      <c r="Q39" s="15"/>
+    </row>
+    <row r="40" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
       <c r="F40" s="5"/>
       <c r="G40" s="9"/>
-      <c r="H40" s="93" t="s">
-        <v>63</v>
-      </c>
-      <c r="I40" s="59"/>
-      <c r="J40" s="49"/>
-      <c r="K40" s="49"/>
-      <c r="L40" s="49"/>
-      <c r="M40" s="52"/>
+      <c r="H40" s="92" t="s">
+        <v>67</v>
+      </c>
+      <c r="I40" s="58"/>
+      <c r="J40" s="48"/>
+      <c r="K40" s="48"/>
+      <c r="L40" s="48"/>
+      <c r="M40" s="51"/>
       <c r="N40" s="9"/>
-      <c r="O40" s="14"/>
-      <c r="P40" s="57"/>
-      <c r="Q40" s="16"/>
-    </row>
-    <row r="41" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B41" s="51" t="s">
+      <c r="O40" s="13"/>
+      <c r="P40" s="8"/>
+      <c r="Q40" s="15"/>
+    </row>
+    <row r="41" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="C41" s="51" t="s">
+      <c r="C41" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="D41" s="115" t="s">
+      <c r="D41" s="112" t="s">
         <v>15</v>
       </c>
-      <c r="E41" s="116"/>
-      <c r="F41" s="117"/>
+      <c r="E41" s="113"/>
+      <c r="F41" s="114"/>
       <c r="G41" s="9"/>
-      <c r="H41" s="94" t="s">
-        <v>64</v>
-      </c>
-      <c r="I41" s="97"/>
-      <c r="J41" s="84"/>
-      <c r="K41" s="84"/>
-      <c r="L41" s="84"/>
-      <c r="M41" s="85"/>
+      <c r="H41" s="93" t="s">
+        <v>68</v>
+      </c>
+      <c r="I41" s="96"/>
+      <c r="J41" s="83"/>
+      <c r="K41" s="83"/>
+      <c r="L41" s="83"/>
+      <c r="M41" s="84"/>
       <c r="N41" s="9"/>
-      <c r="O41" s="14"/>
-      <c r="P41" s="57"/>
-      <c r="Q41" s="16"/>
-    </row>
-    <row r="42" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B42" s="41"/>
-      <c r="C42" s="41"/>
-      <c r="D42" s="108"/>
-      <c r="E42" s="109"/>
-      <c r="F42" s="110"/>
+      <c r="O41" s="13"/>
+      <c r="P41" s="8"/>
+      <c r="Q41" s="15"/>
+    </row>
+    <row r="42" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="40"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="105"/>
+      <c r="E42" s="106"/>
+      <c r="F42" s="62"/>
       <c r="G42" s="9"/>
-      <c r="H42" s="94" t="s">
-        <v>65</v>
-      </c>
-      <c r="I42" s="46"/>
-      <c r="J42" s="42"/>
-      <c r="K42" s="42"/>
-      <c r="L42" s="42"/>
-      <c r="M42" s="48"/>
+      <c r="H42" s="93" t="s">
+        <v>69</v>
+      </c>
+      <c r="I42" s="45"/>
+      <c r="J42" s="41"/>
+      <c r="K42" s="41"/>
+      <c r="L42" s="41"/>
+      <c r="M42" s="47"/>
       <c r="N42" s="9"/>
-      <c r="O42" s="14"/>
-      <c r="P42" s="57"/>
-      <c r="Q42" s="16"/>
-    </row>
-    <row r="43" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B43" s="41"/>
-      <c r="C43" s="88"/>
-      <c r="D43" s="108"/>
-      <c r="E43" s="109"/>
-      <c r="F43" s="110"/>
+      <c r="O42" s="13"/>
+      <c r="P42" s="8"/>
+      <c r="Q42" s="15"/>
+    </row>
+    <row r="43" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="40"/>
+      <c r="C43" s="87"/>
+      <c r="D43" s="105"/>
+      <c r="E43" s="106"/>
+      <c r="F43" s="62"/>
       <c r="G43" s="9"/>
-      <c r="H43" s="95" t="s">
-        <v>88</v>
-      </c>
-      <c r="I43" s="101" t="s">
-        <v>72</v>
-      </c>
-      <c r="J43" s="102"/>
-      <c r="K43" s="102"/>
-      <c r="L43" s="102"/>
-      <c r="M43" s="103"/>
+      <c r="H43" s="94" t="s">
+        <v>90</v>
+      </c>
+      <c r="I43" s="100" t="s">
+        <v>76</v>
+      </c>
+      <c r="J43" s="101"/>
+      <c r="K43" s="101"/>
+      <c r="L43" s="101"/>
+      <c r="M43" s="102"/>
       <c r="N43" s="9"/>
-      <c r="O43" s="14"/>
-      <c r="P43" s="57"/>
-      <c r="Q43" s="16"/>
-    </row>
-    <row r="44" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B44" s="41"/>
-      <c r="C44" s="88"/>
-      <c r="D44" s="108"/>
-      <c r="E44" s="109"/>
-      <c r="F44" s="110"/>
+      <c r="O43" s="13"/>
+      <c r="P43" s="8"/>
+      <c r="Q43" s="15"/>
+    </row>
+    <row r="44" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="40"/>
+      <c r="C44" s="87"/>
+      <c r="D44" s="105"/>
+      <c r="E44" s="106"/>
+      <c r="F44" s="62"/>
       <c r="G44" s="9"/>
-      <c r="H44" s="94" t="s">
-        <v>89</v>
-      </c>
-      <c r="I44" s="46" t="s">
-        <v>51</v>
-      </c>
-      <c r="J44" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="K44" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="L44" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="M44" s="48" t="s">
-        <v>51</v>
-      </c>
+      <c r="H44" s="93" t="s">
+        <v>91</v>
+      </c>
+      <c r="I44" s="45"/>
+      <c r="J44" s="41"/>
+      <c r="K44" s="41"/>
+      <c r="L44" s="41"/>
+      <c r="M44" s="47"/>
       <c r="N44" s="9"/>
-      <c r="O44" s="13"/>
-      <c r="P44" s="57"/>
-      <c r="Q44" s="12"/>
-    </row>
-    <row r="45" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B45" s="41"/>
-      <c r="C45" s="41"/>
-      <c r="D45" s="108"/>
-      <c r="E45" s="109"/>
-      <c r="F45" s="110"/>
+      <c r="O44" s="12"/>
+      <c r="P44" s="5"/>
+      <c r="Q44" s="11"/>
+    </row>
+    <row r="45" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="40"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="105"/>
+      <c r="E45" s="106"/>
+      <c r="F45" s="62"/>
       <c r="G45" s="9"/>
-      <c r="H45" s="94" t="s">
-        <v>92</v>
-      </c>
-      <c r="I45" s="46"/>
-      <c r="J45" s="42"/>
-      <c r="K45" s="42"/>
-      <c r="L45" s="42"/>
-      <c r="M45" s="48"/>
+      <c r="H45" s="93" t="s">
+        <v>94</v>
+      </c>
+      <c r="I45" s="45"/>
+      <c r="J45" s="41"/>
+      <c r="K45" s="41"/>
+      <c r="L45" s="41"/>
+      <c r="M45" s="47"/>
       <c r="N45" s="9"/>
       <c r="O45" s="9"/>
       <c r="P45" s="9"/>
       <c r="Q45" s="9"/>
     </row>
-    <row r="46" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B46" s="41"/>
-      <c r="C46" s="41"/>
-      <c r="D46" s="108"/>
-      <c r="E46" s="109"/>
-      <c r="F46" s="110"/>
+    <row r="46" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="40"/>
+      <c r="C46" s="40"/>
+      <c r="D46" s="105"/>
+      <c r="E46" s="106"/>
+      <c r="F46" s="62"/>
       <c r="G46" s="9"/>
-      <c r="H46" s="95" t="s">
-        <v>90</v>
-      </c>
-      <c r="I46" s="101" t="s">
-        <v>73</v>
-      </c>
-      <c r="J46" s="102"/>
-      <c r="K46" s="102"/>
-      <c r="L46" s="102"/>
-      <c r="M46" s="103"/>
+      <c r="H46" s="94" t="s">
+        <v>92</v>
+      </c>
+      <c r="I46" s="100" t="s">
+        <v>77</v>
+      </c>
+      <c r="J46" s="101"/>
+      <c r="K46" s="101"/>
+      <c r="L46" s="101"/>
+      <c r="M46" s="102"/>
       <c r="N46" s="9"/>
       <c r="O46" s="9"/>
       <c r="P46" s="9"/>
       <c r="Q46" s="9"/>
     </row>
-    <row r="47" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="41"/>
-      <c r="C47" s="41"/>
-      <c r="D47" s="108"/>
-      <c r="E47" s="109"/>
-      <c r="F47" s="110"/>
+    <row r="47" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="40"/>
+      <c r="C47" s="40"/>
+      <c r="D47" s="105"/>
+      <c r="E47" s="106"/>
+      <c r="F47" s="62"/>
       <c r="G47" s="9"/>
-      <c r="H47" s="94" t="s">
-        <v>66</v>
-      </c>
-      <c r="I47" s="46"/>
-      <c r="J47" s="42"/>
-      <c r="K47" s="42"/>
-      <c r="L47" s="42"/>
-      <c r="M47" s="48"/>
+      <c r="H47" s="93" t="s">
+        <v>70</v>
+      </c>
+      <c r="I47" s="45"/>
+      <c r="J47" s="41"/>
+      <c r="K47" s="41"/>
+      <c r="L47" s="41"/>
+      <c r="M47" s="47"/>
       <c r="N47" s="9"/>
       <c r="O47" s="9" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="P47" s="9"/>
       <c r="Q47" s="9"/>
     </row>
-    <row r="48" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B48" s="28" t="s">
+    <row r="48" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="C48" s="41">
+      <c r="C48" s="40">
         <f>SUM(C42:C47)</f>
         <v>0</v>
       </c>
@@ -2983,24 +2963,24 @@
       <c r="E48" s="9"/>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
-      <c r="H48" s="94" t="s">
-        <v>67</v>
-      </c>
-      <c r="I48" s="46"/>
-      <c r="J48" s="42"/>
-      <c r="K48" s="42"/>
-      <c r="L48" s="42"/>
-      <c r="M48" s="48"/>
+      <c r="H48" s="93" t="s">
+        <v>71</v>
+      </c>
+      <c r="I48" s="45"/>
+      <c r="J48" s="41"/>
+      <c r="K48" s="41"/>
+      <c r="L48" s="41"/>
+      <c r="M48" s="47"/>
       <c r="N48" s="9"/>
       <c r="O48" s="9"/>
       <c r="P48" s="9"/>
       <c r="Q48" s="9"/>
     </row>
-    <row r="49" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B49" s="28" t="s">
+    <row r="49" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="C49" s="41">
+      <c r="C49" s="40">
         <f>SUM(C48,C37)</f>
         <v>0</v>
       </c>
@@ -3008,48 +2988,48 @@
       <c r="E49" s="9"/>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
-      <c r="H49" s="94" t="s">
-        <v>68</v>
-      </c>
-      <c r="I49" s="98"/>
-      <c r="J49" s="86"/>
-      <c r="K49" s="86"/>
-      <c r="L49" s="86"/>
-      <c r="M49" s="87"/>
+      <c r="H49" s="93" t="s">
+        <v>72</v>
+      </c>
+      <c r="I49" s="97"/>
+      <c r="J49" s="85"/>
+      <c r="K49" s="85"/>
+      <c r="L49" s="85"/>
+      <c r="M49" s="86"/>
       <c r="N49" s="9"/>
-      <c r="O49" s="42"/>
-      <c r="P49" s="64"/>
-      <c r="Q49" s="42"/>
-    </row>
-    <row r="50" spans="2:18" ht="13.15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B50" s="28"/>
-      <c r="C50" s="43"/>
+      <c r="O49" s="41"/>
+      <c r="P49" s="63"/>
+      <c r="Q49" s="41"/>
+    </row>
+    <row r="50" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="27"/>
+      <c r="C50" s="42"/>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
-      <c r="H50" s="96" t="s">
-        <v>91</v>
-      </c>
-      <c r="I50" s="79"/>
-      <c r="J50" s="80"/>
-      <c r="K50" s="80"/>
-      <c r="L50" s="80"/>
-      <c r="M50" s="81"/>
+      <c r="H50" s="95" t="s">
+        <v>93</v>
+      </c>
+      <c r="I50" s="78"/>
+      <c r="J50" s="79"/>
+      <c r="K50" s="79"/>
+      <c r="L50" s="79"/>
+      <c r="M50" s="80"/>
       <c r="N50" s="9"/>
-      <c r="O50" s="43" t="s">
+      <c r="O50" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="P50" s="43" t="s">
+      <c r="P50" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="Q50" s="43" t="s">
+      <c r="Q50" s="42" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="51" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B51" s="28"/>
-      <c r="C51" s="43"/>
+    <row r="51" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B51" s="27"/>
+      <c r="C51" s="42"/>
       <c r="D51" s="9"/>
       <c r="E51" s="9"/>
       <c r="F51" s="9"/>
@@ -3065,7 +3045,7 @@
       <c r="P51" s="9"/>
       <c r="Q51" s="9"/>
     </row>
-    <row r="52" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B52" s="9"/>
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
@@ -3083,56 +3063,56 @@
       <c r="P52" s="9"/>
       <c r="Q52" s="9"/>
     </row>
-    <row r="53" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B53" s="111"/>
-      <c r="C53" s="111"/>
-      <c r="D53" s="111"/>
-      <c r="E53" s="111" t="s">
-        <v>59</v>
-      </c>
-      <c r="F53" s="111"/>
-      <c r="G53" s="111"/>
-      <c r="H53" s="111"/>
-      <c r="I53" s="111" t="s">
-        <v>69</v>
-      </c>
-      <c r="J53" s="111"/>
-      <c r="K53" s="111"/>
-      <c r="L53" s="111"/>
-      <c r="O53" s="126" t="s">
-        <v>93</v>
-      </c>
-      <c r="P53" s="126"/>
-      <c r="Q53" s="126"/>
-    </row>
-    <row r="54" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B54" s="111" t="s">
-        <v>60</v>
-      </c>
-      <c r="C54" s="111"/>
-      <c r="D54" s="111"/>
-      <c r="E54" s="126" t="s">
+    <row r="53" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B53" s="108"/>
+      <c r="C53" s="108"/>
+      <c r="D53" s="108"/>
+      <c r="E53" s="108" t="s">
+        <v>63</v>
+      </c>
+      <c r="F53" s="108"/>
+      <c r="G53" s="108"/>
+      <c r="H53" s="108"/>
+      <c r="I53" s="108" t="s">
+        <v>73</v>
+      </c>
+      <c r="J53" s="108"/>
+      <c r="K53" s="108"/>
+      <c r="L53" s="108"/>
+      <c r="O53" s="123" t="s">
+        <v>95</v>
+      </c>
+      <c r="P53" s="123"/>
+      <c r="Q53" s="123"/>
+    </row>
+    <row r="54" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B54" s="108" t="s">
+        <v>64</v>
+      </c>
+      <c r="C54" s="108"/>
+      <c r="D54" s="108"/>
+      <c r="E54" s="123" t="s">
+        <v>79</v>
+      </c>
+      <c r="F54" s="123"/>
+      <c r="G54" s="123"/>
+      <c r="H54" s="123"/>
+      <c r="I54" s="108" t="s">
+        <v>74</v>
+      </c>
+      <c r="J54" s="108"/>
+      <c r="K54" s="108"/>
+      <c r="L54" s="108"/>
+      <c r="N54" t="s">
+        <v>65</v>
+      </c>
+      <c r="O54" s="108" t="s">
         <v>75</v>
       </c>
-      <c r="F54" s="126"/>
-      <c r="G54" s="126"/>
-      <c r="H54" s="126"/>
-      <c r="I54" s="111" t="s">
-        <v>70</v>
-      </c>
-      <c r="J54" s="111"/>
-      <c r="K54" s="111"/>
-      <c r="L54" s="111"/>
-      <c r="N54" t="s">
-        <v>61</v>
-      </c>
-      <c r="O54" s="111" t="s">
-        <v>71</v>
-      </c>
-      <c r="P54" s="111"/>
-      <c r="Q54" s="111"/>
-    </row>
-    <row r="55" spans="2:18" ht="54.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P54" s="108"/>
+      <c r="Q54" s="108"/>
+    </row>
+    <row r="55" spans="2:18" ht="54.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B55" s="9"/>
       <c r="C55" s="9"/>
       <c r="D55" s="9"/>
@@ -3140,23 +3120,19 @@
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
       <c r="H55" s="9"/>
-      <c r="I55" s="118" t="s">
-        <v>76</v>
-      </c>
-      <c r="J55" s="118"/>
-      <c r="K55" s="118"/>
-      <c r="L55" s="118"/>
-      <c r="M55" s="78"/>
+      <c r="I55" s="115"/>
+      <c r="J55" s="115"/>
+      <c r="K55" s="115"/>
+      <c r="L55" s="115"/>
+      <c r="M55" s="77"/>
       <c r="N55" s="9"/>
-      <c r="O55" s="118" t="s">
-        <v>77</v>
-      </c>
-      <c r="P55" s="118"/>
-      <c r="Q55" s="118"/>
-      <c r="R55" s="78"/>
-    </row>
-    <row r="58" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="E58" s="65"/>
+      <c r="O55" s="115"/>
+      <c r="P55" s="115"/>
+      <c r="Q55" s="115"/>
+      <c r="R55" s="77"/>
+    </row>
+    <row r="58" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="E58" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="34">
@@ -3175,24 +3151,24 @@
     <mergeCell ref="E54:H54"/>
     <mergeCell ref="I54:L54"/>
     <mergeCell ref="I55:L55"/>
-    <mergeCell ref="D45:F45"/>
     <mergeCell ref="O54:Q54"/>
-    <mergeCell ref="D44:F44"/>
     <mergeCell ref="B54:D54"/>
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D43:F43"/>
     <mergeCell ref="D41:F41"/>
-    <mergeCell ref="D46:F46"/>
     <mergeCell ref="B53:D53"/>
-    <mergeCell ref="D47:F47"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D47:E47"/>
     <mergeCell ref="I31:M31"/>
     <mergeCell ref="I34:M34"/>
     <mergeCell ref="I43:M43"/>
     <mergeCell ref="I46:M46"/>
     <mergeCell ref="D33:E33"/>
     <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D42:F42"/>
     <mergeCell ref="D32:E32"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
@@ -3206,7 +3182,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9D6F89B-2F67-41D8-AAA8-9E96940477A2}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
@@ -3217,7 +3193,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E74AD6C-8D0B-4421-9E6A-635D6611049A}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>

</xml_diff>